<commit_message>
feat: simplify item imports and large quote expansion
- replace dense CSV/Excel guidance with a three-step bilingual flow and plain-language errors

- refresh the static Excel template instructions, comments, and validation prompts without changing its import format

- show progress feedback while expanding large quotations

- extend component, performance, and template parser coverage
</commit_message>
<xml_diff>
--- a/file/templates/quotation-line-items-template.xlsx
+++ b/file/templates/quotation-line-items-template.xlsx
@@ -15,8 +15,6 @@
   <definedNames>
     <definedName name="QuantityUnits">'_Lists'!$A$2:$A$17</definedName>
     <definedName name="CurrencyCodes">'_Lists'!$B$2:$B$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Import Data'!$A$1:$J$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Examples 示例'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -123,7 +121,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -159,11 +157,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00B4C6E7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -197,6 +201,15 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -281,62 +294,62 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Hierarchy code such as 1, 1.1, or 1.1.1. Blank creates a new top-level item.
-层级编号，例如 1、1.1 或 1.1.1。留空会创建新的一级明细。</t>
+        <t>Sets the level: 1, 1.1, or 1.1.1. Blank creates a new top-level item.
+表示层级：1、1.1 或 1.1.1。留空会自动新建一级项目。</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Required text for every item row.
-每个明细行都必须填写。</t>
+        <t>Item name. Required on every row.
+项目名称，每一行都要填。</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Optional description text.
-可选的说明文字。</t>
+        <t>Optional description.
+项目说明，可以不填。</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Plain number above 0. Required for leaf rows; a blank group quantity defaults to 1.
-大于 0 的普通数字。叶子行必填；父级留空时默认为 1。</t>
+        <t>Quantity above 0. Required when the item has no sub-items; otherwise blank becomes 1.
+数量，必须大于 0。没有子项时必填；有子项时留空会自动使用 1。</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Unit text such as EA, set, hour, or day. Blank defaults to EA.
-单位，例如 EA、set、hour 或 day。留空默认为 EA。</t>
+        <t>Unit such as EA, set, hour, or day. Blank becomes EA.
+单位，例如 EA、set、hour 或 day。留空会自动使用 EA。</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Manual selling price above 0. When filled, it controls sales pricing.
-大于 0 的手动售价。填写后由该值控制销售定价。</t>
+        <t>Direct selling price above 0. Leave blank when using cost + markup.
+直接填写的售价，必须大于 0。按成本加价时留空。</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Required above 0 for cost-plus leaves. Optional non-negative analysis cost for manual pricing.
-成本加价叶子行必须大于 0；手动定价时可填写非负分析成本。</t>
+        <t>Required above 0 for cost + markup. Optional for a directly priced item.
+按成本加价时必填且必须大于 0。直接报价时可以不填。</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Three-letter currency code. Required for cost-plus leaves.
-三位货币代码。成本加价叶子行必填。</t>
+        <t>Three-letter cost currency such as USD or CNY. Required for cost + markup.
+三位成本币种，例如 USD 或 CNY。按成本加价时必填。</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Optional existing tax-class ID or label from the quotation.
-可选；必须填写报价中已有的税类 ID 或名称。</t>
+        <t>Tax name or ID already used in the quotation. Blank uses the parent/default.
+当前报价里已有的税率名称或 ID。留空就使用上级或默认税率。</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Enter percentage points from 0 to 1000. Enter 15 for 15%; do not apply Excel Percentage format.
-填写 0 到 1000 的百分点。15% 请填写 15；不要使用 Excel 百分比格式。</t>
+        <t>Enter 15 for 15%. Do not apply Excel Percentage format.
+加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
       </text>
     </comment>
   </commentList>
@@ -351,80 +364,80 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Hierarchy code such as 1, 1.1, or 1.1.1. Blank creates a new top-level item.
-层级编号，例如 1、1.1 或 1.1.1。留空会创建新的一级明细。</t>
+        <t>Sets the level: 1, 1.1, or 1.1.1. Blank creates a new top-level item.
+表示层级：1、1.1 或 1.1.1。留空会自动新建一级项目。</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Required text for every item row.
-每个明细行都必须填写。</t>
+        <t>Item name. Required on every row.
+项目名称，每一行都要填。</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Optional description text.
-可选的说明文字。</t>
+        <t>Optional description.
+项目说明，可以不填。</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Plain number above 0. Required for leaf rows; a blank group quantity defaults to 1.
-大于 0 的普通数字。叶子行必填；父级留空时默认为 1。</t>
+        <t>Quantity above 0. Required when the item has no sub-items; otherwise blank becomes 1.
+数量，必须大于 0。没有子项时必填；有子项时留空会自动使用 1。</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Unit text such as EA, set, hour, or day. Blank defaults to EA.
-单位，例如 EA、set、hour 或 day。留空默认为 EA。</t>
+        <t>Unit such as EA, set, hour, or day. Blank becomes EA.
+单位，例如 EA、set、hour 或 day。留空会自动使用 EA。</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Manual selling price above 0. When filled, it controls sales pricing.
-大于 0 的手动售价。填写后由该值控制销售定价。</t>
+        <t>Direct selling price above 0. Leave blank when using cost + markup.
+直接填写的售价，必须大于 0。按成本加价时留空。</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Required above 0 for cost-plus leaves. Optional non-negative analysis cost for manual pricing.
-成本加价叶子行必须大于 0；手动定价时可填写非负分析成本。</t>
+        <t>Required above 0 for cost + markup. Optional for a directly priced item.
+按成本加价时必填且必须大于 0。直接报价时可以不填。</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Three-letter currency code. Required for cost-plus leaves.
-三位货币代码。成本加价叶子行必填。</t>
+        <t>Three-letter cost currency such as USD or CNY. Required for cost + markup.
+三位成本币种，例如 USD 或 CNY。按成本加价时必填。</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Optional existing tax-class ID or label from the quotation.
-可选；必须填写报价中已有的税类 ID 或名称。</t>
+        <t>Tax name or ID already used in the quotation. Blank uses the parent/default.
+当前报价里已有的税率名称或 ID。留空就使用上级或默认税率。</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Enter percentage points from 0 to 1000. Enter 15 for 15%; do not apply Excel Percentage format.
-填写 0 到 1000 的百分点。15% 请填写 15；不要使用 Excel 百分比格式。</t>
+        <t>Enter 15 for 15%. Do not apply Excel Percentage format.
+加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
       </text>
     </comment>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Group row: children determine price; markup may be inherited.
-父级行：价格由子项汇总；加价率可被继承。</t>
+        <t>This item has sub-items 1.1 and 1.2, so its total comes from those rows.
+这个项目下面有 1.1 和 1.2，金额会从这两行合计。</t>
       </text>
     </comment>
     <comment ref="A3" authorId="0" shapeId="0">
       <text>
-        <t>Cost-plus leaf: unit_cost and cost_currency are required.
-成本加价叶子行：unit_cost 和 cost_currency 必填。</t>
+        <t>Cost + markup: cost is 1200 USD and markup is 15%.
+按成本加价：成本是 1200 USD，加价率是 15%。</t>
       </text>
     </comment>
     <comment ref="A4" authorId="0" shapeId="0">
       <text>
-        <t>Manual-price leaf: manual_unit_price controls sales; unit_cost is optional analysis data.
-手动定价叶子行：manual_unit_price 控制销售定价；unit_cost 是可选分析数据。</t>
+        <t>Direct price: selling price is 500 per day. The 100 USD cost is optional analysis data.
+直接报价：售价是每天 500。100 USD 成本只用于可选分析。</t>
       </text>
     </comment>
   </commentList>
@@ -774,261 +787,249 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Quotation Line-Item Import Workbook / 报价明细导入工作簿</t>
+          <t>Quotation Item Import Template / 报价项目导入模板</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>The app imports this .xlsx workbook directly from the exact “Import Data” sheet. CSV UTF-8 remains supported. / 应用可从名称完全为“Import Data”的工作表直接导入此 .xlsx 工作簿，同时仍支持 CSV UTF-8。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Only fill the “Import Data” sheet. Keep its name and first-row headers unchanged. / 只填写“Import Data”工作表，工作表名称和第一行表头都不要改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>English workflow</t>
+          <t>Three steps</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>中文流程</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>1. Read the rules below, then open the “Import Data” sheet.</t>
+          <t>只要三步</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>1. Open “Import Data”. Fill one item per row.</t>
         </is>
       </c>
       <c r="B6" s="14" t="n"/>
       <c r="C6" s="14" t="n"/>
       <c r="D6" s="14" t="n"/>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>1. 阅读下方规则，然后打开“Import Data”工作表。</t>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>1. 打开“Import Data”，每行填一个项目。</t>
         </is>
       </c>
       <c r="F6" s="14" t="n"/>
       <c r="G6" s="14" t="n"/>
       <c r="H6" s="14" t="n"/>
     </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2. Keep the 10 English headers. Enter one group or leaf item per row.</t>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>2. Use item_code values 1, 1.1, and 1.1.1 to set the level.</t>
         </is>
       </c>
       <c r="B7" s="14" t="n"/>
       <c r="C7" s="14" t="n"/>
       <c r="D7" s="14" t="n"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>2. 保留 10 个英文表头，每行填写一个父级或叶子明细。</t>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>2. item_code 用 1、1.1、1.1.1 表示层级。</t>
         </is>
       </c>
       <c r="F7" s="14" t="n"/>
       <c r="G7" s="14" t="n"/>
       <c r="H7" s="14" t="n"/>
     </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>3. Use item_code values such as 1, 1.1, and 1.1.1 to define hierarchy.</t>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>3. Save as .xlsx. In the app, choose Import Excel, check the result, and confirm.</t>
         </is>
       </c>
       <c r="B8" s="14" t="n"/>
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="14" t="n"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>3. 使用 1、1.1、1.1.1 这类 item_code 定义层级。</t>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>3. 保存为 .xlsx，在软件里选择“导入 Excel”，检查结果后确认。</t>
         </is>
       </c>
       <c r="F8" s="14" t="n"/>
       <c r="G8" s="14" t="n"/>
       <c r="H8" s="14" t="n"/>
     </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>4. Save as .xlsx without renaming “Import Data” or changing its row-one headers. For CSV, export that sheet as CSV UTF-8.</t>
-        </is>
-      </c>
+    <row r="9" ht="8" customHeight="1">
+      <c r="A9" s="16" t="n"/>
       <c r="B9" s="14" t="n"/>
       <c r="C9" s="14" t="n"/>
       <c r="D9" s="14" t="n"/>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>4. 保存为 .xlsx，且不要重命名“Import Data”或修改第一行表头。如需 CSV，请将该工作表导出为 CSV UTF-8。</t>
-        </is>
-      </c>
+      <c r="E9" s="16" t="n"/>
       <c r="F9" s="14" t="n"/>
       <c r="G9" s="14" t="n"/>
       <c r="H9" s="14" t="n"/>
     </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>5. In the app, choose Import line items, then Choose Excel or Choose CSV. Review the report and confirm the import.</t>
-        </is>
-      </c>
+    <row r="10" ht="8" customHeight="1">
+      <c r="A10" s="15" t="n"/>
       <c r="B10" s="14" t="n"/>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>5. 在应用中选择“导入明细”，再选择 Excel 或 CSV。检查导入报告，然后确认导入。</t>
-        </is>
-      </c>
+      <c r="E10" s="15" t="n"/>
       <c r="F10" s="14" t="n"/>
       <c r="G10" s="14" t="n"/>
       <c r="H10" s="14" t="n"/>
     </row>
-    <row r="13">
+    <row r="11" ht="8" customHeight="1"/>
+    <row r="12" ht="8" customHeight="1"/>
+    <row r="13" ht="24" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Rules and precedence</t>
+          <t>How to fill prices</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>规则和优先级</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="50" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Required by role: every row needs item_name. Leaves also need qty. Cost-plus leaves need unit_cost and cost_currency; manual-price leaves need manual_unit_price.</t>
+          <t>价格怎么填</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Has sub-items: fill item_name. The total comes from the rows below.</t>
         </is>
       </c>
       <c r="B14" s="14" t="n"/>
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="14" t="n"/>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>按行类型必填：每行都需要 item_name。叶子行还需要 qty；成本加价叶子行需要 unit_cost 和 cost_currency；手动定价叶子行需要 manual_unit_price。</t>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>有子项：填写 item_name，金额会从下面的子项合计。</t>
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
       <c r="G14" s="14" t="n"/>
       <c r="H14" s="14" t="n"/>
     </row>
-    <row r="15" ht="50" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Numbers: use plain decimals. No currency symbols, thousands separators, hexadecimal, NaN, infinity, or scientific notation.</t>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Cost + markup: fill item_name, qty, unit_cost, and cost_currency.</t>
         </is>
       </c>
       <c r="B15" s="14" t="n"/>
       <c r="C15" s="14" t="n"/>
       <c r="D15" s="14" t="n"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>数字：只使用普通小数。不要填写货币符号、千位分隔符、十六进制、NaN、无穷大或科学计数法。</t>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>按成本加价：填写 item_name、qty、unit_cost 和 cost_currency。</t>
         </is>
       </c>
       <c r="F15" s="14" t="n"/>
       <c r="G15" s="14" t="n"/>
       <c r="H15" s="14" t="n"/>
     </row>
-    <row r="16" ht="50" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Markup: enter 15 for 15%. Keep markup_override as a normal number from 0 to 1000; do not apply Excel Percentage format.</t>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Direct price: fill item_name, qty, and manual_unit_price. unit_cost is optional.</t>
         </is>
       </c>
       <c r="B16" s="14" t="n"/>
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>加价率：15% 请填写 15。markup_override 必须是 0 到 1000 的普通数字，不要设置为 Excel 百分比格式。</t>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>直接填写售价：填写 item_name、qty 和 manual_unit_price。unit_cost 可以不填。</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
       <c r="G16" s="14" t="n"/>
       <c r="H16" s="14" t="n"/>
     </row>
-    <row r="17" ht="50" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Pricing: manual_unit_price selects manual pricing and controls sales. If blank, a leaf uses cost-plus and needs unit_cost and cost_currency. With manual pricing, unit_cost is optional analysis data. Group price, cost, and currency are ignored.</t>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Before importing</t>
         </is>
       </c>
       <c r="B17" s="14" t="n"/>
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="14" t="n"/>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>定价：填写 manual_unit_price 即选择手动定价并控制销售价格；留空时叶子行使用成本加价，并需要 unit_cost 和 cost_currency。手动定价时 unit_cost 仅为可选分析数据。父级价格、成本和币种会忽略。</t>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>导入前看一眼</t>
         </is>
       </c>
       <c r="F17" s="14" t="n"/>
       <c r="G17" s="14" t="n"/>
       <c r="H17" s="14" t="n"/>
     </row>
-    <row r="18" ht="50" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Inheritance: a leaf tax class or markup overrides its parent/default. Group tax class and markup may be inherited.</t>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Use plain numbers. Do not use formulas, currency symbols, commas, or scientific notation.</t>
         </is>
       </c>
       <c r="B18" s="14" t="n"/>
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>继承：叶子行税类或加价率优先于父级/默认值；父级税类和加价率可被继承。</t>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>只填普通数字，不要使用公式、货币符号、千位逗号或科学计数法。</t>
         </is>
       </c>
       <c r="F18" s="14" t="n"/>
       <c r="G18" s="14" t="n"/>
       <c r="H18" s="14" t="n"/>
     </row>
-    <row r="19" ht="50" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Tax classes: tax_class must match an existing quotation tax-class ID or label. This static workbook cannot provide that dropdown.</t>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>For 15% markup, enter 15. Do not apply Excel Percentage format.</t>
         </is>
       </c>
       <c r="B19" s="14" t="n"/>
       <c r="C19" s="14" t="n"/>
       <c r="D19" s="14" t="n"/>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>税类：tax_class 必须匹配当前报价已有的税类 ID 或名称。静态工作簿无法提供该下拉列表。</t>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
       <c r="G19" s="14" t="n"/>
       <c r="H19" s="14" t="n"/>
     </row>
-    <row r="20" ht="50" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Safety: examples are on a separate sheet. Do not save or import the Examples sheet.</t>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>tax_class must match a tax name or ID in the current quotation. Leave blank to use the parent/default.</t>
         </is>
       </c>
       <c r="B20" s="14" t="n"/>
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>安全：示例位于单独工作表。不要保存或导入 Examples 示例工作表。</t>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>tax_class 必须和当前报价里的税率名称或 ID 一致；留空就使用上级或默认税率。</t>
         </is>
       </c>
       <c r="F20" s="14" t="n"/>
       <c r="G20" s="14" t="n"/>
       <c r="H20" s="14" t="n"/>
     </row>
+    <row r="21" ht="8" customHeight="1"/>
+    <row r="22" ht="8" customHeight="1"/>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Header colors / 表头颜色：  Required / 必填     Conditional / 按行类型必填     Optional / 可选</t>
+          <t>Header colors / 表头颜色：  Required / 必填     Sometimes required / 有时必填     Optional / 可选</t>
         </is>
       </c>
     </row>
@@ -1375,22 +1376,22 @@
     </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Item name required / 必须填写项目名称" error="Enter item_name when this row contains data. / 本行有数据时必须填写 item_name。" promptTitle="Item name required / 必须填写名称" prompt="Enter item_name for every used row. / 每个已使用行都必须填写 item_name。" type="custom" errorStyle="stop">
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Item name required / 项目名称必填" error="If this row has data, enter item_name. / 这一行有内容时，必须填写 item_name。" promptTitle="Item name required / 项目名称必填" prompt="Enter item_name on every used row. / 每个有内容的行都要填写 item_name。" type="custom" errorStyle="stop">
       <formula1>OR(COUNTA($A2:$J2)=0,LEN(TRIM($B2))&gt;0)</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Quantity above zero / 数量必须大于 0" error="Leave blank only for a group; leaves require qty above 0. / 仅父级可留空；叶子行数量必须大于 0。" promptTitle="Quantity above zero / 数量必须大于 0" prompt="Leave blank only for a group; leaves require qty above 0. / 仅父级可留空；叶子行数量必须大于 0。" type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Quantity above 0 / 数量必须大于 0" error="Leave blank only when the item has sub-items; otherwise enter qty above 0. / 只有下面有子项时才能留空；否则 qty 必须大于 0。" promptTitle="Quantity above 0 / 数量必须大于 0" prompt="Leave blank only when the item has sub-items; otherwise enter qty above 0. / 只有下面有子项时才能留空；否则 qty 必须大于 0。" type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Manual price above zero / 手动价格必须大于 0" error="Leave blank for cost-plus pricing. / 成本加价定价时留空。" promptTitle="Manual price above zero / 手动价格必须大于 0" prompt="Leave blank for cost-plus pricing. / 成本加价定价时留空。" type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="F2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Direct price above 0 / 直接售价必须大于 0" error="Leave blank when using cost + markup. / 按成本加价时留空。" promptTitle="Direct price above 0 / 直接售价必须大于 0" prompt="Enter a direct selling price, or leave blank for cost + markup. / 直接报价时填写售价；按成本加价时留空。" type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Cost cannot be negative / 成本不能为负数" error="Cost-plus leaves require a cost above 0. / 成本加价叶子行的成本必须大于 0。" promptTitle="Cost cannot be negative / 成本不能为负数" prompt="Cost-plus leaves require a cost above 0. / 成本加价叶子行的成本必须大于 0。" type="decimal" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="G2:G1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Cost cannot be negative / 成本不能是负数" error="Cost + markup requires unit_cost above 0. Directly priced items may leave it blank. / 按成本加价时 unit_cost 必须大于 0；直接报价时可以留空。" promptTitle="Cost for pricing or analysis / 定价或分析成本" prompt="Required for cost + markup; optional for a directly priced item. / 按成本加价时必填；直接报价时可以不填。" type="decimal" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Suggested currency / 建议币种" error="Choose a common code or continue with another supported three-letter code. / 可选择常用代码，也可继续填写其他受支持的三位代码。" promptTitle="Suggested currency / 建议币种" prompt="Choose a common code or continue with another supported three-letter code. / 可选择常用代码，也可继续填写其他受支持的三位代码。" type="list" errorStyle="warning">
+    <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Cost currency / 成本币种" error="Pick a common code or type another supported three-letter code. / 请选择常用代码，或填写软件支持的其他三位代码。" promptTitle="Cost currency / 成本币种" prompt="Pick a common code or type another supported three-letter code. / 请选择常用代码，或填写软件支持的其他三位代码。" type="list" errorStyle="warning">
       <formula1>=CurrencyCodes</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Markup 0 to 1000 / 加价率范围 0 到 1000" error="Enter 15 for 15%. Do not use Excel Percentage format. / 15% 请填写 15，不要使用 Excel 百分比格式。" promptTitle="Markup 0 to 1000 / 加价率范围 0 到 1000" prompt="Enter 15 for 15%. Do not use Excel Percentage format. / 15% 请填写 15，不要使用 Excel 百分比格式。" type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Markup 0 to 1000 / 加价率 0 到 1000" error="Enter 15 for 15%. Do not apply Excel Percentage format. / 15% 就填 15，不要套用 Excel 的百分比格式。" promptTitle="Markup 0 to 1000 / 加价率 0 到 1000" prompt="Enter 15 for 15%. Do not apply Excel Percentage format. / 15% 就填 15，不要套用 Excel 的百分比格式。" type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1000</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(quotations): improve line-item scaling and summary controls
- virtualize large root and child item lists while preserving focused-row reveal
- synchronize summary views and cache descendant pricing lazily
- keep bulk expansion one-shot so manual nested state survives tree edits
- clarify optional markup overrides in bilingual and Excel import guidance
- expand performance and regression coverage
</commit_message>
<xml_diff>
--- a/file/templates/quotation-line-items-template.xlsx
+++ b/file/templates/quotation-line-items-template.xlsx
@@ -934,10 +934,10 @@
       <c r="G15" s="14" t="n"/>
       <c r="H15" s="14" t="n"/>
     </row>
-    <row r="16" ht="40" customHeight="1">
+    <row r="16" ht="140" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Direct price: fill item_name, qty, and manual_unit_price. unit_cost is optional.</t>
+          <t>Direct price: enter manual_unit_price when you already know what to charge the customer—for example, the exact cost is unknown, you received a fixed price, or you know this price will cover the cost. The system will use it directly. To calculate from cost + markup instead, leave it blank and enter unit_cost and cost_currency. Enter markup_override only when this row needs a different markup; otherwise leave it blank to inherit the parent or quotation default.</t>
         </is>
       </c>
       <c r="B16" s="14" t="n"/>
@@ -945,7 +945,7 @@
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>直接填写售价：填写 item_name、qty 和 manual_unit_price。unit_cost 可以不填。</t>
+          <t>直接填写售价：已经知道要报给客户的单价时，填写 manual_unit_price。例如：暂时不知道具体成本、拿到的是一口价，或者确定这个售价足以覆盖成本。填写后系统会直接使用这个售价。如果需要按“成本 + 加价率”计算，请留空，并填写 unit_cost 和 cost_currency。只有该行需要单独加价率时才填写 markup_override；否则留空，使用上级或报价默认值。</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>

</xml_diff>

<commit_message>
Refresh line item Excel template
</commit_message>
<xml_diff>
--- a/file/templates/quotation-line-items-template.xlsx
+++ b/file/templates/quotation-line-items-template.xlsx
@@ -342,14 +342,14 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Tax name or ID already used in the quotation. Blank uses the parent/default.
-当前报价里已有的税率名称或 ID。留空就使用上级或默认税率。</t>
+        <t>Enter 15 for 15%. Do not apply Excel Percentage format.
+加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Enter 15 for 15%. Do not apply Excel Percentage format.
-加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
+        <t>Tax name or ID already used in the quotation. Blank uses the parent/default.
+当前报价里已有的税率名称或 ID。留空就使用上级或默认税率。</t>
       </text>
     </comment>
   </commentList>
@@ -412,32 +412,14 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Tax name or ID already used in the quotation. Blank uses the parent/default.
-当前报价里已有的税率名称或 ID。留空就使用上级或默认税率。</t>
+        <t>Enter 15 for 15%. Do not apply Excel Percentage format.
+加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Enter 15 for 15%. Do not apply Excel Percentage format.
-加价率 15% 就填 15，不要套用 Excel 的百分比格式。</t>
-      </text>
-    </comment>
-    <comment ref="A2" authorId="0" shapeId="0">
-      <text>
-        <t>This item has sub-items 1.1 and 1.2, so its total comes from those rows.
-这个项目下面有 1.1 和 1.2，金额会从这两行合计。</t>
-      </text>
-    </comment>
-    <comment ref="A3" authorId="0" shapeId="0">
-      <text>
-        <t>Cost + markup: cost is 1200 USD and markup is 15%.
-按成本加价：成本是 1200 USD，加价率是 15%。</t>
-      </text>
-    </comment>
-    <comment ref="A4" authorId="0" shapeId="0">
-      <text>
-        <t>Direct price: selling price is 500 per day. The 100 USD cost is optional analysis data.
-直接报价：售价是每天 500。100 USD 成本只用于可选分析。</t>
+        <t>Tax name or ID already used in the quotation. Blank uses the parent/default.
+当前报价里已有的税率名称或 ID。留空就使用上级或默认税率。</t>
       </text>
     </comment>
   </commentList>
@@ -456,16 +438,16 @@
     <tableColumn id="6" name="manual_unit_price"/>
     <tableColumn id="7" name="unit_cost"/>
     <tableColumn id="8" name="cost_currency"/>
-    <tableColumn id="9" name="tax_class"/>
-    <tableColumn id="10" name="markup_override"/>
+    <tableColumn id="9" name="markup_override"/>
+    <tableColumn id="10" name="tax_class"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExampleDataTable" displayName="ExampleDataTable" ref="A1:J4" headerRowCount="1">
-  <autoFilter ref="A1:J4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExampleDataTable" displayName="ExampleDataTable" ref="A1:J13" headerRowCount="1">
+  <autoFilter ref="A1:J13"/>
   <tableColumns count="10">
     <tableColumn id="1" name="item_code"/>
     <tableColumn id="2" name="item_name"/>
@@ -475,8 +457,8 @@
     <tableColumn id="6" name="manual_unit_price"/>
     <tableColumn id="7" name="unit_cost"/>
     <tableColumn id="8" name="cost_currency"/>
-    <tableColumn id="9" name="tax_class"/>
-    <tableColumn id="10" name="markup_override"/>
+    <tableColumn id="9" name="markup_override"/>
+    <tableColumn id="10" name="tax_class"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -771,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1024,20 +1006,48 @@
       <c r="G20" s="14" t="n"/>
       <c r="H20" s="14" t="n"/>
     </row>
-    <row r="21" ht="8" customHeight="1"/>
-    <row r="22" ht="8" customHeight="1"/>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Header colors / 表头颜色：  Required / 必填     Sometimes required / 有时必填     Optional / 可选</t>
-        </is>
-      </c>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Foreign cost currencies: set their exchange rates in the quotation after import.</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>外币成本：导入后在报价中设置对应汇率。</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="14" t="n"/>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Blank markup uses the nearest parent rate, then the quotation default.</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>加价率留空：先继承最近的上级，否则使用报价默认值。</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="14" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="34">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="E16:H16"/>
     <mergeCell ref="E7:H7"/>
@@ -1045,8 +1055,10 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E22:H22"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="E18:H18"/>
+    <mergeCell ref="E21:H21"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="E14:H14"/>
@@ -1058,11 +1070,11 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="E19:H19"/>
-    <mergeCell ref="A23:H23"/>
     <mergeCell ref="E10:H10"/>
     <mergeCell ref="E13:H13"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="E9:H9"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="E6:H6"/>
     <mergeCell ref="E15:H15"/>
     <mergeCell ref="A14:D14"/>
@@ -1306,8 +1318,8 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1353,12 +1365,12 @@
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
+          <t>markup_override</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
           <t>tax_class</t>
-        </is>
-      </c>
-      <c r="J1" s="8" t="inlineStr">
-        <is>
-          <t>markup_override</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1403,7 @@
     <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Cost currency / 成本币种" error="Pick a common code or type another supported three-letter code. / 请选择常用代码，或填写软件支持的其他三位代码。" promptTitle="Cost currency / 成本币种" prompt="Pick a common code or type another supported three-letter code. / 请选择常用代码，或填写软件支持的其他三位代码。" type="list" errorStyle="warning">
       <formula1>=CurrencyCodes</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Markup 0 to 1000 / 加价率 0 到 1000" error="Enter 15 for 15%. Do not apply Excel Percentage format. / 15% 就填 15，不要套用 Excel 的百分比格式。" promptTitle="Markup 0 to 1000 / 加价率 0 到 1000" prompt="Enter 15 for 15%. Do not apply Excel Percentage format. / 15% 就填 15，不要套用 Excel 的百分比格式。" type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Markup 0 to 1000 / 加价率 0 到 1000" error="Enter 15 for 15%. Do not apply Excel Percentage format. / 15% 就填 15，不要套用 Excel 的百分比格式。" promptTitle="Markup 0 to 1000 / 加价率 0 到 1000" prompt="Enter 15 for 15%. Do not apply Excel Percentage format. / 15% 就填 15，不要套用 Excel 的百分比格式。" type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1000</formula2>
     </dataValidation>
@@ -1410,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1421,8 +1433,11 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="3" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1468,12 +1483,22 @@
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
+          <t>markup_override</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
           <t>tax_class</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
-        <is>
-          <t>markup_override</t>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Row / 行</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>What it shows / 说明</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1510,12 @@
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>Equipment package / 设备包</t>
+          <t>Pump Skid / 泵组撬装系统</t>
         </is>
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
-          <t>Supply and commissioning / 供货和调试</t>
+          <t>Complete package / 成套系统</t>
         </is>
       </c>
       <c r="D2" s="12" t="n">
@@ -1504,9 +1529,19 @@
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
       <c r="H2" s="12" t="n"/>
-      <c r="I2" s="12" t="n"/>
-      <c r="J2" s="12" t="n">
-        <v>10</v>
+      <c r="I2" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="J2" s="12" t="n"/>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>Parent rollup; child fallback 18% / 父项汇总；子项默认 18%</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1517,7 +1552,7 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Pump / 泵</t>
+          <t>Mechanical / 机械设备</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
@@ -1526,56 +1561,48 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>set</t>
         </is>
       </c>
       <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="G3" s="12" t="n"/>
+      <c r="H3" s="12" t="n"/>
       <c r="I3" s="12" t="n"/>
-      <c r="J3" s="12" t="n">
-        <v>15</v>
-      </c>
+      <c r="J3" s="12" t="n"/>
+      <c r="L3" s="16" t="n"/>
+      <c r="M3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>Commissioning / 调试</t>
+          <t>Centrifugal Pump / 离心泵</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>On-site work / 现场工作</t>
+          <t>Process pump / 工艺泵</t>
         </is>
       </c>
       <c r="D4" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>500</v>
-      </c>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="n"/>
       <c r="G4" s="12" t="n">
-        <v>100</v>
+        <v>1200</v>
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
@@ -1584,6 +1611,398 @@
       </c>
       <c r="I4" s="12" t="n"/>
       <c r="J4" s="12" t="n"/>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>USD cost; inherits 18% / USD 成本；继承 18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>1.1.2</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Electric Motor / 电机</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>High-efficiency motor / 高效电机</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" s="12" t="n">
+        <v>6800</v>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="J5" s="12" t="n"/>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>1.1.2</t>
+        </is>
+      </c>
+      <c r="M5" s="16" t="inlineStr">
+        <is>
+          <t>CNY cost; leaf override 25% / CNY 成本；本行覆盖为 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Controls / 控制系统</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Panel and drives / 控制柜及驱动</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>Nested child fallback 12% / 下级子项默认 12%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>1.2.1</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>PLC Panel / PLC 控制柜</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Main control panel / 主控制柜</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
+      <c r="L7" s="16" t="n"/>
+      <c r="M7" s="16" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>1.2.2</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Drive / 变频器</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Motor drive / 电机驱动</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>1.2.3</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Control Cable / 控制电缆</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Shielded cable / 屏蔽电缆</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>1.2.3</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>EUR cost; explicit 0% / EUR 成本；明确 0% 加价</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Services / 服务</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Site services / 现场服务</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Commissioning / 调试</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>On-site work / 现场工作</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Manual price with USD cost / 直接售价并记录 USD 成本</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Training / 培训</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Operator training / 操作培训</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>800</v>
+      </c>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+      <c r="M12" s="15" t="inlineStr">
+        <is>
+          <t>Manual price without cost / 直接售价，不记录成本</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Export Packing / 出口包装</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Seaworthy packing / 适海包装</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n">
+        <v>2800</v>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>Uses quotation default markup / 使用报价默认加价率</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>